<commit_message>
feat: add On Hold status, actual dates, charts dashboard, and date parsing fixes
- New TaskStatus: On Hold (only In Progress cards can move here)
- Auto-set Actual Start Date on Todo→In Progress, Actual End Date on →Done
- On Hold modal captures reason; On Hold Date auto-set
- On Hold badge shown on TaskCard; On Hold Log report sub-tab
- Charts dashboard: KPI cards, status donut, workload stacked bar,
  sprint burndown, velocity, cycle time, planned vs actual, on-hold impact
- Recharts loaded client-side only (ssr:false) to prevent SSR crash
- Fixed burndown infinite loop caused by non-ISO date strings in Excel
- parseDate now normalises human-readable dates (e.g. "Jun 24, 2026") to ISO
- de-sprints.xlsx and sample-tasks.xlsx updated with new columns
- Dynamic sheet tab name used as page title
</commit_message>
<xml_diff>
--- a/public/de-sprints.xlsx
+++ b/public/de-sprints.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:N17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,9 +422,24 @@
         <v>End Date</v>
       </c>
       <c r="H1" t="str">
+        <v>Actual Start Date</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Actual End Date</v>
+      </c>
+      <c r="J1" t="str">
+        <v>On Hold Date</v>
+      </c>
+      <c r="K1" t="str">
+        <v>On Hold Reason</v>
+      </c>
+      <c r="L1" t="str">
         <v>Blocked By</v>
       </c>
-      <c r="I1" t="str">
+      <c r="M1" t="str">
+        <v>Dependency</v>
+      </c>
+      <c r="N1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -436,7 +451,7 @@
         <v>PMIX</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D2" t="str">
         <v>Norman</v>
@@ -448,12 +463,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G2" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v/>
       </c>
     </row>
@@ -465,7 +495,7 @@
         <v>SKP</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D3" t="str">
         <v>Norman</v>
@@ -477,12 +507,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G3" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v/>
       </c>
     </row>
@@ -494,7 +539,7 @@
         <v>SKP PRs</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D4" t="str">
         <v>Norman</v>
@@ -506,12 +551,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G4" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>T1</v>
+      </c>
+      <c r="N4" t="str">
         <v/>
       </c>
     </row>
@@ -523,7 +583,7 @@
         <v>Store Copilot</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D5" t="str">
         <v>Norman</v>
@@ -535,12 +595,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G5" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
         <v/>
       </c>
     </row>
@@ -552,7 +627,7 @@
         <v>Sec Assessment for BT for chowking</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D6" t="str">
         <v>Norman</v>
@@ -564,12 +639,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G6" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
         <v/>
       </c>
     </row>
@@ -581,7 +671,7 @@
         <v>Store copilot usage dashboard</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D7" t="str">
         <v>Norman</v>
@@ -593,12 +683,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G7" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
         <v/>
       </c>
     </row>
@@ -610,7 +715,7 @@
         <v>DAM</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D8" t="str">
         <v>Norman</v>
@@ -622,12 +727,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G8" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
         <v/>
       </c>
     </row>
@@ -639,7 +759,7 @@
         <v>MIPNL</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D9" t="str">
         <v>JMR</v>
@@ -651,12 +771,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G9" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
         <v/>
       </c>
     </row>
@@ -668,7 +803,7 @@
         <v>SOS JPOS</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D10" t="str">
         <v>JMR</v>
@@ -680,12 +815,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G10" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
         <v/>
       </c>
     </row>
@@ -697,7 +847,7 @@
         <v>Project Birthday</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D11" t="str">
         <v>JMR</v>
@@ -709,12 +859,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G11" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
         <v/>
       </c>
     </row>
@@ -726,7 +891,7 @@
         <v>Operation Execelence</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D12" t="str">
         <v>JMR</v>
@@ -738,12 +903,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G12" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
         <v/>
       </c>
     </row>
@@ -755,7 +935,7 @@
         <v>QMAI</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D13" t="str">
         <v>Nel</v>
@@ -767,12 +947,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G13" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
         <v/>
       </c>
     </row>
@@ -784,7 +979,7 @@
         <v>Komunidad</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D14" t="str">
         <v>Nel</v>
@@ -796,12 +991,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G14" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
         <v/>
       </c>
     </row>
@@ -813,24 +1023,39 @@
         <v>Twillio</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D15" t="str">
         <v>Nel</v>
       </c>
       <c r="E15" t="str">
-        <v>Todo</v>
+        <v>On Hold</v>
       </c>
       <c r="F15" t="str">
         <v>2026-06-15</v>
       </c>
       <c r="G15" t="str">
-        <v>Jun 24, 2026</v>
+        <v>2026-06-24</v>
       </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
         <v/>
       </c>
     </row>
@@ -842,7 +1067,7 @@
         <v>CRM UCG</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D16" t="str">
         <v>Nel</v>
@@ -854,12 +1079,27 @@
         <v>2026-06-15</v>
       </c>
       <c r="G16" t="str">
-        <v>Jun 23, 2026</v>
+        <v>2026-06-23</v>
       </c>
       <c r="H16" t="str">
         <v/>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
         <v/>
       </c>
     </row>
@@ -871,7 +1111,7 @@
         <v>QM Qualtrics</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>tbfo</v>
       </c>
       <c r="D17" t="str">
         <v>Nel</v>
@@ -883,18 +1123,33 @@
         <v>2026-06-15</v>
       </c>
       <c r="G17" t="str">
-        <v>Jun 19, 2026</v>
+        <v>2026-06-19</v>
       </c>
       <c r="H17" t="str">
         <v/>
       </c>
       <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>